<commit_message>
feat(command): add smart help-based verification for new options
- Add _is_help_verification_needed() to detect new option/parameter mentions
- Add _extract_base_command() to extract base command for --help usage
- Add validate_command_with_help() to verify options in --help output
- Modify validate_command() to use --help when new options are mentioned
- Fix table header parsing to only read first row as headers
- Add test_commands_with_options.html with option test cases

This allows validating new command options by checking --help output
instead of executing potentially dangerous commands.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/output/command_report.xlsx
+++ b/document/output/command_report.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -487,27 +487,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5.1 进程相关命令对比</t>
+          <t>5.1 命令选项新增验证</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>检查内核版本</t>
+          <t>检查timedatectl命令</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>uname -r</t>
+          <t>timedatectl</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>版本升级到5.10</t>
+          <t>新增revert选项</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>影响驱动兼容性</t>
+          <t>支持恢复时区设置</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -520,27 +520,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>5.1 进程相关命令对比</t>
+          <t>5.1 命令选项新增验证</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>检查Java版本</t>
+          <t>检查systemctl命令</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>java -version 2&gt;&amp;1 | head -1</t>
+          <t>systemctl</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>从JDK 8升级到JDK 11</t>
+          <t>新增edit选项</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>影响应用兼容性</t>
+          <t>支持编辑unit文件</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -553,27 +553,27 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>5.2 配置文件检查</t>
+          <t>5.1 命令选项新增验证</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>检查SSH配置</t>
+          <t>检查firewall-cmd命令</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>grep "^Port" /etc/ssh/sshd_config</t>
+          <t>firewall-cmd</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>端口从22改为2222</t>
+          <t>增加info选项</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>影响远程连接</t>
+          <t>查看防火墙信息</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -586,27 +586,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>5.2 配置文件检查</t>
+          <t>5.2 其他命令变更</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>检查数据库版本</t>
+          <t>检查内核版本</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>mysql --version</t>
+          <t>uname -r</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>从5.7升级到8.0</t>
+          <t>版本升级到5.10</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>影响SQL语法</t>
+          <t>影响驱动兼容性</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -615,6 +615,39 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5.2 其他命令变更</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>检查Java版本</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>java -version 2&gt;&amp;1 | head -1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>从JDK 8升级到JDK 11</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>影响应用兼容性</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>